<commit_message>
Addition of energy transfers
</commit_message>
<xml_diff>
--- a/src/fluorophores/cy5_properties.xlsx
+++ b/src/fluorophores/cy5_properties.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwuerzburg-my.sharepoint.com/personal/vincent_ebert_stud-mail_uni-wuerzburg_de/Documents/GitHub/Photoswitching/src/fluorophores/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_AD4DB114E441178AC67DF44A5610C320683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDF55206-A1C9-41ED-B83A-EC0E7509C56E}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="11_AD4DB114E441178AC67DF44A5610C320683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93C94ADF-3D06-44DB-8FB2-19CF753EDE20}"/>
   <bookViews>
-    <workbookView xWindow="45972" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="45972" yWindow="4908" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>maximum extinction coefficient [1/(cm M)]</t>
   </si>
@@ -61,6 +61,12 @@
   </si>
   <si>
     <t>quantum yield</t>
+  </si>
+  <si>
+    <t>fret spectral overlap integral</t>
+  </si>
+  <si>
+    <t>fret dipole orientation factor</t>
   </si>
 </sst>
 </file>
@@ -127,10 +133,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -396,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="39.86328125" bestFit="1" customWidth="1"/>
@@ -500,6 +502,25 @@
         <v>1.6999999999999999E-17</v>
       </c>
     </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="2">
+        <v>0.66666599999999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="B14" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="597" r:id="rId1"/>

</xml_diff>